<commit_message>
Fix synthetic data quality: seasonal achievement, retention, Gebyur, part_name
- Add monthly achievement narrative (Jan O/T low A/T high, Apr-May post-Eid
  dip, Aug dip, Oct-Dec peak) with yearly total ~103-105%
- Add customer activity types (loyal/regular/occasional/rare) for realistic
  retention & churn patterns (82% retention vs previous ~100%)
- Add part_name column to part_master.xlsx, fixing Cross-sell/Diversifikasi
  KeyError on Part_Name
- Add SO_Type "C" + Campaign_Code for ~8% TMO orders, fixing empty Gebyur tab
- Remove ODOM tab from Customer page (all synthetic = non-ODOM)
- Remove 6 broken tabs from Operasional Partnumber (Claim, Goodwill,
  Lead Time, Fill Rate, Status Fulfillment, Substitusi)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TASTI_SYNTHETIC/Pno7KP.xlsx
+++ b/TASTI_SYNTHETIC/Pno7KP.xlsx
@@ -431,55 +431,55 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>39N924M458</t>
+          <t>49U399D862</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Electrical</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>77E770F344</t>
+          <t>21R786E528</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Suspension</t>
+          <t>Electrical</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18D185X686</t>
+          <t>22Q151G393</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Engine Oil</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>24H971S301</t>
+          <t>73X237B995</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Engine Oil</t>
+          <t>Electrical</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>80E327V183</t>
+          <t>41E182F976</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -491,31 +491,31 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>59Q949R141</t>
+          <t>40M772T789</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Engine Oil</t>
+          <t>Suspension</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>73U316W414</t>
+          <t>12F586B304</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Accessories</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>46G618C307</t>
+          <t>45W529Z366</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -527,103 +527,103 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>75Y551N287</t>
+          <t>96S927A253</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Engine Oil</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>78S376A389</t>
+          <t>94L149H588</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>69B811H684</t>
+          <t>82W678F194</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Body Parts</t>
+          <t>Accessories</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>71A605G837</t>
+          <t>68R398W621</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Body Parts</t>
+          <t>Brake Parts</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>53F482U278</t>
+          <t>40E279A801</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Body Parts</t>
+          <t>Suspension</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>78D231Y259</t>
+          <t>73T113M963</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Brake Parts</t>
+          <t>Filter</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>27Y969X767</t>
+          <t>15L907K894</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Body Parts</t>
+          <t>Brake Parts</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>52L658U471</t>
+          <t>57V593G150</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Engine Oil</t>
+          <t>Electrical</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>77Q565V469</t>
+          <t>70F835W363</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -635,91 +635,91 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>91Y820P893</t>
+          <t>82H242Y590</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Filter</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>48D535E581</t>
+          <t>63F450V637</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Engine Oil</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>19Q566T131</t>
+          <t>67X872R901</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Suspension</t>
+          <t>Accessories</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>23J216E866</t>
+          <t>61P604D548</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Brake Parts</t>
+          <t>Accessories</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>96C631C305</t>
+          <t>67L211F801</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Suspension</t>
+          <t>Filter</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>60F583W255</t>
+          <t>79N377Q312</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Engine Oil</t>
+          <t>Filter</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>20R641T976</t>
+          <t>74U441S656</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Filter</t>
+          <t>Brake Parts</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>69V126M730</t>
+          <t>46R128B862</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -731,19 +731,19 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>84L285C888</t>
+          <t>45K580Y957</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Filter</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>91K777N691</t>
+          <t>97Y627H501</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -755,7 +755,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>54U918S131</t>
+          <t>64D462X328</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -767,31 +767,31 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>77T254V670</t>
+          <t>47K646X730</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Engine Oil</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>76C717D713</t>
+          <t>63N297N716</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Filter</t>
+          <t>Electrical</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>37N876P812</t>
+          <t>73C531C832</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -803,43 +803,43 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>31V197X765</t>
+          <t>86H552Q765</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Suspension</t>
+          <t>Filter</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>84E883T177</t>
+          <t>77X387K618</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Engine Oil</t>
+          <t>Electrical</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>91J659A895</t>
+          <t>73R395L967</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>84M630B711</t>
+          <t>44S180Q769</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -851,343 +851,343 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>14Y783D166</t>
+          <t>96K328Q670</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Filter</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>18P660B955</t>
+          <t>73P148A469</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Accessories</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>38Y870X295</t>
+          <t>12Z541Y716</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Suspension</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>17G962Z172</t>
+          <t>81N182T928</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Suspension</t>
+          <t>Accessories</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>55Y457P391</t>
+          <t>58F976G849</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Body Parts</t>
+          <t>Engine Oil</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>83Z803N519</t>
+          <t>84N822X760</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Engine Oil</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>60G387D173</t>
+          <t>74J485B149</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Brake Parts</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>87B671W656</t>
+          <t>79L137F416</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Suspension</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>25K223J232</t>
+          <t>83C717R896</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Suspension</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>93S124V273</t>
+          <t>32F281B706</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Suspension</t>
+          <t>Brake Parts</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>29W181U500</t>
+          <t>93J452W723</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Engine Oil</t>
+          <t>Electrical</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>28S796Z590</t>
+          <t>32N133X733</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Suspension</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>47C648X574</t>
+          <t>73J218E680</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Body Parts</t>
+          <t>Brake Parts</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>50X382P769</t>
+          <t>92S776W448</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Brake Parts</t>
+          <t>Filter</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>60Y285E480</t>
+          <t>64W737P863</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Suspension</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>89L218K963</t>
+          <t>37N358Y580</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Engine Oil</t>
+          <t>Electrical</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>13X668Z623</t>
+          <t>44T632M601</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Brake Parts</t>
+          <t>Accessories</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>52N105K497</t>
+          <t>85P440L610</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>38B790F133</t>
+          <t>70Z186V901</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Filter</t>
+          <t>Electrical</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>71J223B266</t>
+          <t>84N838B423</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Suspension</t>
+          <t>Filter</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>23A433V455</t>
+          <t>43K359P654</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Engine Oil</t>
+          <t>Suspension</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>36W960M806</t>
+          <t>96Q332D906</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Brake Parts</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>83N966R507</t>
+          <t>57M624X879</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Suspension</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>29Y732T634</t>
+          <t>16M768T328</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Suspension</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>19Q107Y707</t>
+          <t>97P770Z553</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Suspension</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>13K855U244</t>
+          <t>19J756V360</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Engine Oil</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>70Y738J607</t>
+          <t>56B477H382</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Body Parts</t>
+          <t>Engine Oil</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>81F409T245</t>
+          <t>19K823Y952</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Body Parts</t>
+          <t>Filter</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>25Y141Y586</t>
+          <t>69B485S440</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1199,151 +1199,151 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>73N660Y104</t>
+          <t>92H891F411</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Filter</t>
+          <t>Electrical</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>41U897M115</t>
+          <t>87B337W776</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Accessories</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>32S210F120</t>
+          <t>96E654F696</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Brake Parts</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>25Q403X156</t>
+          <t>95M390K208</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Body Parts</t>
+          <t>Accessories</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>42U752R449</t>
+          <t>45E231P273</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Filter</t>
+          <t>Suspension</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>85U563Z744</t>
+          <t>74L163C435</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Brake Parts</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>20M444D783</t>
+          <t>87H350T124</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Filter</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>83F370F899</t>
+          <t>76M702H671</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Engine Oil</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>38Z966N121</t>
+          <t>95E895B381</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Body Parts</t>
+          <t>Accessories</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>64N417G347</t>
+          <t>22R558U231</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Body Parts</t>
+          <t>Accessories</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>24Y937V205</t>
+          <t>27L337P307</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Engine Oil</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>77G451B326</t>
+          <t>56R464Q393</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Suspension</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>30U333X367</t>
+          <t>29F753A207</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -1355,127 +1355,127 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>40U618J784</t>
+          <t>24D608B140</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Body Parts</t>
+          <t>Suspension</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>25V110F191</t>
+          <t>39N818V805</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Electrical</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>78B583F623</t>
+          <t>12E542A580</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Suspension</t>
+          <t>Engine Oil</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>91E126K414</t>
+          <t>46Z424P553</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Body Parts</t>
+          <t>Suspension</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>91A800B878</t>
+          <t>67B258E762</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Brake Parts</t>
+          <t>Engine Oil</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>46U413C361</t>
+          <t>50S258F367</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Electrical</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>90L584Y930</t>
+          <t>90P522Z401</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Engine Oil</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>15L565G585</t>
+          <t>87F378Q620</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Filter</t>
+          <t>Engine Oil</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>29D845X603</t>
+          <t>74X815A709</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Brake Parts</t>
+          <t>Engine Oil</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>29T950W466</t>
+          <t>55H236P657</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Engine Oil</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>86W115P529</t>
+          <t>26G247V709</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -1487,175 +1487,175 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>46A649W573</t>
+          <t>36F697N550</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>52Z382K617</t>
+          <t>94R195J698</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Suspension</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>50U355E268</t>
+          <t>64K709T907</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Brake Parts</t>
+          <t>Suspension</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>41Y346W246</t>
+          <t>87T523H493</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Engine Oil</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>61J862F863</t>
+          <t>61D734T498</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Suspension</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>54Z328A135</t>
+          <t>20M143E672</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Accessories</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>68G188G572</t>
+          <t>73Z912F946</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Filter</t>
+          <t>Electrical</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>20X960H253</t>
+          <t>83G823L368</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Body Parts</t>
+          <t>Filter</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>61K533B854</t>
+          <t>57R563Z131</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Brake Parts</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>58C567D876</t>
+          <t>42L154G702</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Suspension</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>36Z698H634</t>
+          <t>97M582E376</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Filter</t>
+          <t>Engine Oil</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>66F625B819</t>
+          <t>70W837T790</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Filter</t>
+          <t>Accessories</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>31D224H171</t>
+          <t>58Q247M586</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Filter</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>34B424K717</t>
+          <t>53K940K321</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Brake Parts</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>16U380C296</t>
+          <t>60S519X212</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>26G875D769</t>
+          <t>90V294B764</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -1679,103 +1679,103 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>37K794U382</t>
+          <t>55U303L649</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Engine Oil</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>65R737L558</t>
+          <t>27T154B395</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Engine Oil</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>58Z259N967</t>
+          <t>73U794H923</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Brake Parts</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>43N962E327</t>
+          <t>53N846J226</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Engine Oil</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>73F426J882</t>
+          <t>77F507T569</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Filter</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>17U859N118</t>
+          <t>40W170R346</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Suspension</t>
+          <t>Electrical</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>69V958F630</t>
+          <t>56Z686F690</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Engine Oil</t>
+          <t>Electrical</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>50T704B234</t>
+          <t>31G163C220</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>24Q523K778</t>
+          <t>10W364G868</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -1787,103 +1787,103 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>12C840J750</t>
+          <t>97H525R136</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Suspension</t>
+          <t>Engine Oil</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>45J404C403</t>
+          <t>85T808S329</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Filter</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>41L706Z812</t>
+          <t>66F290L185</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Engine Oil</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>75Q631J504</t>
+          <t>75G721C468</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Engine Oil</t>
+          <t>Brake Parts</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>25A139B241</t>
+          <t>39B553G685</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Suspension</t>
+          <t>Electrical</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>64D306D397</t>
+          <t>24L312T914</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Brake Parts</t>
+          <t>Accessories</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>34M449S469</t>
+          <t>50D571W916</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Filter</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>52U604V741</t>
+          <t>97W575P162</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Engine Oil</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>41U842C151</t>
+          <t>81D707Q543</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -1895,163 +1895,163 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>37T405A708</t>
+          <t>33X522S648</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Engine Oil</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>72N148E767</t>
+          <t>90Z603Z817</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Accessories</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>13Q711N389</t>
+          <t>28Q472X142</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Body Parts</t>
+          <t>Brake Parts</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>19F540G508</t>
+          <t>63F416W427</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Brake Parts</t>
+          <t>Engine Oil</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>57Q493C657</t>
+          <t>41E185V152</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Electrical</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>79A509G922</t>
+          <t>48P763Z436</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Suspension</t>
+          <t>Engine Oil</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>42H991S513</t>
+          <t>82Z492C536</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Filter</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>28X150B127</t>
+          <t>97Y195W199</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Brake Parts</t>
+          <t>Accessories</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>49L153N369</t>
+          <t>89V924U181</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>71A540Y782</t>
+          <t>55X693W912</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Filter</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>47S229U778</t>
+          <t>25D871S921</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Accessories</t>
+          <t>Body Parts</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>57B882T410</t>
+          <t>59B257Z511</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Accessories</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>67B846Q378</t>
+          <t>38A884P434</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Suspension</t>
+          <t>Electrical</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>64K665K693</t>
+          <t>26P115W528</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -2063,7 +2063,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>70L953W917</t>
+          <t>84Z132L329</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">

</xml_diff>